<commit_message>
chore(jdt) : update jdt
</commit_message>
<xml_diff>
--- a/docs/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\ReadME-MAUI\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1542BEB0-45D3-4B9E-A7FA-68813A3EC093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8962861-ED93-40A0-A5FF-9E111BB09E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3390" yWindow="2100" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="4080" yWindow="2790" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="47">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -148,22 +148,40 @@
     <t>Faire la maquette de la page livre</t>
   </si>
   <si>
-    <t>Création du projet, et versionning du projet</t>
+    <t>WIP</t>
   </si>
   <si>
-    <t>Ajout du grid (place holders) pour les livres sur la page d'accueil</t>
+    <t>Analyse du cahier des charges</t>
   </si>
   <si>
-    <t>Renseignement sur le fonctionnement des fichiers .epub</t>
+    <t>Conception UI/UX : maquettage de l'écran d'accueil (bibliothèque).</t>
   </si>
   <si>
-    <t>Importation d'un fichier epub utilisant la librarie VersOne</t>
+    <t>Conception UI/UX : maquettage de la vue détaillée d'un ouvrage.</t>
   </si>
   <si>
-    <t>Ajout d'une classe Book et structure qui permet de sauvegarder les données chargé en ram</t>
+    <t>Initialisation de l'environnement de développement et du dépôt git.</t>
   </si>
   <si>
-    <t>WIP</t>
+    <t>Implémentation de la grille d'affichage dynamique avec placeholders.</t>
+  </si>
+  <si>
+    <t>Étude technique de la structure et du parsing des fichiers .epub.</t>
+  </si>
+  <si>
+    <t>Intégration de la librairie VersOne et test d'importation de fichiers epub</t>
+  </si>
+  <si>
+    <t>Modélisation de la classe "Book" et gestion de la persistance en RAM.</t>
+  </si>
+  <si>
+    <t>Finalisation de création de classe, et l'affichage des livres ajoutés suivant la maquette</t>
+  </si>
+  <si>
+    <t>Implémentation de la page d'affichage de contenu d'un livre</t>
+  </si>
+  <si>
+    <t>WIP, à faire le changement des pages</t>
   </si>
 </sst>
 </file>
@@ -1171,10 +1189,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>40</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>340</c:v>
+                  <c:v>570</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2026,10 +2044,10 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.10526315789473684</c:v>
+                  <c:v>9.5238095238095233E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.89473684210526316</c:v>
+                  <c:v>0.90476190476190477</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4270,7 +4288,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>6 heures 20 minutes</v>
+        <v>10 heures 30 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4285,15 +4303,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>260</v>
+        <v>450</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>380</v>
+        <v>630</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4415,13 +4433,13 @@
       </c>
       <c r="C10" s="31"/>
       <c r="D10" s="32">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G10" s="39"/>
       <c r="M10" t="s">
@@ -4437,22 +4455,20 @@
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="63">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="34">
-        <v>46107</v>
-      </c>
-      <c r="C11" s="35">
-        <v>1</v>
-      </c>
+        <v>46099</v>
+      </c>
+      <c r="C11" s="35"/>
       <c r="D11" s="36">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E11" s="37" t="s">
         <v>17</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G11" s="40"/>
       <c r="M11" t="s">
@@ -4468,20 +4484,20 @@
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="62">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="30">
-        <v>46107</v>
+        <v>46099</v>
       </c>
       <c r="C12" s="31"/>
       <c r="D12" s="32">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
@@ -4497,22 +4513,20 @@
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13" s="34">
-        <v>46113</v>
-      </c>
-      <c r="C13" s="35">
-        <v>1</v>
-      </c>
+        <v>46099</v>
+      </c>
+      <c r="C13" s="35"/>
       <c r="D13" s="36">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="E13" s="37" t="s">
         <v>17</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G13" s="40"/>
       <c r="N13">
@@ -4525,24 +4539,24 @@
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="62">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B14" s="30">
-        <v>46143</v>
-      </c>
-      <c r="C14" s="31"/>
+        <v>46107</v>
+      </c>
+      <c r="C14" s="31">
+        <v>1</v>
+      </c>
       <c r="D14" s="32">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E14" s="33" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="G14" s="39" t="s">
         <v>40</v>
       </c>
+      <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
       </c>
@@ -4551,15 +4565,23 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="63" t="str">
+      <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="34"/>
+        <v>13</v>
+      </c>
+      <c r="B15" s="34">
+        <v>46107</v>
+      </c>
       <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+      <c r="D15" s="36">
+        <v>20</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>41</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -4569,61 +4591,101 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="62" t="str">
+      <c r="A16" s="62">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
+        <v>14</v>
+      </c>
+      <c r="B16" s="30">
+        <v>46113</v>
+      </c>
+      <c r="C16" s="31">
+        <v>1</v>
+      </c>
+      <c r="D16" s="32">
+        <v>30</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>42</v>
+      </c>
       <c r="G16" s="39"/>
       <c r="O16">
         <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="63" t="str">
+      <c r="A17" s="63">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="34"/>
+        <v>14</v>
+      </c>
+      <c r="B17" s="34">
+        <v>46113</v>
+      </c>
       <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="40"/>
+      <c r="D17" s="36">
+        <v>50</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" s="40" t="s">
+        <v>35</v>
+      </c>
       <c r="O17">
         <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="62" t="str">
+      <c r="A18" s="62">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="30"/>
+        <v>17</v>
+      </c>
+      <c r="B18" s="30">
+        <v>46134</v>
+      </c>
       <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="23"/>
+      <c r="D18" s="32">
+        <v>40</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>44</v>
+      </c>
       <c r="G18" s="39"/>
       <c r="O18">
         <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="63" t="str">
+      <c r="A19" s="63">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="40"/>
+        <v>17</v>
+      </c>
+      <c r="B19" s="34">
+        <v>46134</v>
+      </c>
+      <c r="C19" s="35">
+        <v>1</v>
+      </c>
+      <c r="D19" s="36">
+        <v>30</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="40" t="s">
+        <v>46</v>
+      </c>
       <c r="O19">
         <v>55</v>
       </c>
@@ -10922,11 +10984,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10934,11 +10996,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>0 h 40 min</v>
+        <v>1 h 00 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.10526315789473684</v>
+        <v>9.5238095238095233E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10955,15 +11017,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>220</v>
+        <v>390</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>340</v>
+        <v>570</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10971,11 +11033,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>5 h 40 min</v>
+        <v>9 h 30 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.89473684210526316</v>
+        <v>0.90476190476190477</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11101,26 +11163,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>260</v>
+        <v>450</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>380</v>
+        <v>630</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>31</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>6 h 20 min</v>
+        <v>10 h 30 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>7.0370370370370375E-2</v>
+        <v>0.11666666666666667</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>31</v>
@@ -11159,12 +11221,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11357,20 +11421,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11395,12 +11460,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore : màj jdt
</commit_message>
<xml_diff>
--- a/docs/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\ReadME-MAUI\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8962861-ED93-40A0-A5FF-9E111BB09E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{000EA077-B7FC-411E-948C-9F1D8478DB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="2790" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="3735" yWindow="2445" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="48">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -182,6 +182,9 @@
   </si>
   <si>
     <t>WIP, à faire le changement des pages</t>
+  </si>
+  <si>
+    <t>WIP, j'essaie de trouver un moyen pour afficher les pages horizontalement en changant les pages avec les boutons</t>
   </si>
 </sst>
 </file>
@@ -1192,7 +1195,7 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>570</c:v>
+                  <c:v>660</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2044,10 +2047,10 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>9.5238095238095233E-2</c:v>
+                  <c:v>8.3333333333333329E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.90476190476190477</c:v>
+                  <c:v>0.91666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4288,7 +4291,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>10 heures 30 minutes</v>
+        <v>12 heures 0 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4303,15 +4306,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>630</v>
+        <v>720</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4690,17 +4693,29 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="62" t="str">
+    <row r="20" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="62">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="39"/>
+        <v>18</v>
+      </c>
+      <c r="B20" s="30">
+        <v>46141</v>
+      </c>
+      <c r="C20" s="31">
+        <v>1</v>
+      </c>
+      <c r="D20" s="32">
+        <v>30</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="39" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="63" t="str">
@@ -11000,7 +11015,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>9.5238095238095233E-2</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11017,15 +11032,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>390</v>
+        <v>420</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>570</v>
+        <v>660</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11033,11 +11048,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>9 h 30 min</v>
+        <v>11 h 00 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.90476190476190477</v>
+        <v>0.91666666666666663</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11163,26 +11178,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>630</v>
+        <v>720</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>31</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>10 h 30 min</v>
+        <v>12 h 00 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.11666666666666667</v>
+        <v>0.13333333333333333</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>31</v>
@@ -11221,17 +11236,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11420,6 +11424,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11430,17 +11445,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11459,6 +11463,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>